<commit_message>
Continued work on booklet.
Mostly focused on week 4 with a few additional updates in other timelines and activities.
</commit_message>
<xml_diff>
--- a/course_revision_progress.xlsx
+++ b/course_revision_progress.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10419"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dhasterok/Documents/GitHub/EART_3017/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC6377F4-E58C-1946-941F-4D06294FBFBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD7539E8-8B0F-BA47-AB87-A8405C5D74BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3100" yWindow="3400" windowWidth="26040" windowHeight="14680" xr2:uid="{4DB3ECE9-6214-0C48-84B8-5529643C9A33}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="92">
   <si>
     <t>Revision progress for geophysics 3A</t>
   </si>
@@ -306,6 +306,12 @@
   </si>
   <si>
     <t>outlined</t>
+  </si>
+  <si>
+    <t>Booklet</t>
+  </si>
+  <si>
+    <t>PPT</t>
   </si>
 </sst>
 </file>
@@ -732,7 +738,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4155229F-2A7B-BB47-BAA3-02BB9B8AE321}">
-  <dimension ref="A1:O37"/>
+  <dimension ref="A1:P37"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="6.5" bestFit="1" customWidth="1"/>
@@ -740,16 +746,22 @@
     <col min="3" max="3" width="14" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="5.83203125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="19.6640625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="8.1640625" customWidth="1"/>
-    <col min="14" max="14" width="31.83203125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.1640625" customWidth="1"/>
+    <col min="15" max="15" width="31.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.2">
       <c r="C1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="I2" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="J2" s="10"/>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A3" s="10" t="s">
         <v>45</v>
       </c>
@@ -768,19 +780,22 @@
         <v>31</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>32</v>
+        <v>90</v>
       </c>
       <c r="J3" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="K3" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="K3" s="5" t="s">
+      <c r="L3" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="M3" s="5" t="s">
+      <c r="N3" s="5" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A4" s="6" t="s">
         <v>49</v>
       </c>
@@ -791,17 +806,17 @@
       <c r="F4" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="K4" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="M4" s="6" t="s">
+      <c r="L4" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="N4" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="N4" s="5" t="s">
+      <c r="O4" s="5" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A5" s="7"/>
       <c r="B5" s="8" t="s">
         <v>1</v>
@@ -827,17 +842,20 @@
       <c r="J5" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="M5" s="6">
+      <c r="K5" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="N5" s="6">
         <v>1</v>
       </c>
-      <c r="N5" t="s">
+      <c r="O5" t="s">
         <v>58</v>
       </c>
-      <c r="O5" s="3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P5" s="3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A6" s="6" t="s">
         <v>2</v>
       </c>
@@ -853,23 +871,24 @@
       <c r="H6" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="I6" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="J6" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="M6" s="6">
+      <c r="I6" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="J6" s="2"/>
+      <c r="K6" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="N6" s="6">
         <v>2</v>
       </c>
-      <c r="N6" t="s">
+      <c r="O6" t="s">
         <v>59</v>
       </c>
-      <c r="O6" s="3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P6" s="3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A7" s="6">
         <v>1</v>
       </c>
@@ -891,23 +910,24 @@
       <c r="H7" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="I7" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="J7" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="M7" s="6">
+      <c r="I7" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="J7" s="2"/>
+      <c r="K7" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="N7" s="6">
         <v>3</v>
       </c>
-      <c r="N7" t="s">
+      <c r="O7" t="s">
         <v>60</v>
       </c>
-      <c r="O7" s="4" t="s">
+      <c r="P7" s="4" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A8" s="6">
         <v>2</v>
       </c>
@@ -921,20 +941,20 @@
       <c r="F8" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="K8" s="2" t="s">
+      <c r="L8" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="M8" s="6">
+      <c r="N8" s="6">
         <v>4</v>
       </c>
-      <c r="N8" t="s">
+      <c r="O8" t="s">
         <v>61</v>
       </c>
-      <c r="O8" s="3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P8" s="3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A9" s="6">
         <v>3</v>
       </c>
@@ -956,23 +976,24 @@
       <c r="H9" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="I9" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="J9" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="M9" s="6">
-        <v>5</v>
-      </c>
-      <c r="N9" t="s">
+      <c r="I9" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="J9" s="2"/>
+      <c r="K9" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="N9" s="6">
+        <v>5</v>
+      </c>
+      <c r="O9" t="s">
         <v>62</v>
       </c>
-      <c r="O9" s="3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P9" s="3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A10" s="6">
         <v>4</v>
       </c>
@@ -994,23 +1015,24 @@
       <c r="H10" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="I10" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="J10" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="M10" s="6">
+      <c r="I10" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="J10" s="2"/>
+      <c r="K10" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="N10" s="6">
         <v>6</v>
       </c>
-      <c r="N10" t="s">
+      <c r="O10" t="s">
         <v>63</v>
       </c>
-      <c r="O10" s="4" t="s">
+      <c r="P10" s="4" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A11" s="6">
         <v>5</v>
       </c>
@@ -1032,23 +1054,24 @@
       <c r="H11" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="I11" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="J11" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="M11" s="6">
-        <v>7</v>
-      </c>
-      <c r="N11" t="s">
+      <c r="I11" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="J11" s="2"/>
+      <c r="K11" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="N11" s="6">
+        <v>7</v>
+      </c>
+      <c r="O11" t="s">
         <v>64</v>
       </c>
-      <c r="O11" s="3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P11" s="3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A12" s="6" t="s">
         <v>3</v>
       </c>
@@ -1064,23 +1087,24 @@
       <c r="H12" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="I12" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="J12" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="M12" s="6">
-        <v>8</v>
-      </c>
-      <c r="N12" t="s">
+      <c r="I12" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="J12" s="2"/>
+      <c r="K12" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="N12" s="6">
+        <v>8</v>
+      </c>
+      <c r="O12" t="s">
         <v>65</v>
       </c>
-      <c r="O12" s="4" t="s">
+      <c r="P12" s="4" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A13" s="6">
         <v>6</v>
       </c>
@@ -1094,20 +1118,20 @@
       <c r="F13" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="K13" s="2" t="s">
+      <c r="L13" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="M13" s="6">
+      <c r="N13" s="6">
         <v>9</v>
       </c>
-      <c r="N13" t="s">
+      <c r="O13" t="s">
         <v>66</v>
       </c>
-      <c r="O13" s="4" t="s">
+      <c r="P13" s="4" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A14" s="6">
         <v>7</v>
       </c>
@@ -1129,23 +1153,24 @@
       <c r="H14" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="I14" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="J14" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="M14" s="6">
+      <c r="I14" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="J14" s="2"/>
+      <c r="K14" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="N14" s="6">
         <v>10</v>
       </c>
-      <c r="N14" t="s">
+      <c r="O14" t="s">
         <v>67</v>
       </c>
-      <c r="O14" s="4" t="s">
+      <c r="P14" s="4" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A15" s="6">
         <v>8</v>
       </c>
@@ -1167,23 +1192,24 @@
       <c r="H15" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="I15" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="J15" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="M15" s="6">
+      <c r="I15" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="J15" s="2"/>
+      <c r="K15" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="N15" s="6">
         <v>11</v>
       </c>
-      <c r="N15" t="s">
+      <c r="O15" t="s">
         <v>68</v>
       </c>
-      <c r="O15" s="3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P15" s="3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A16" s="6">
         <v>9</v>
       </c>
@@ -1205,23 +1231,24 @@
       <c r="H16" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="I16" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="J16" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="M16" s="6">
+      <c r="I16" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="J16" s="2"/>
+      <c r="K16" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="N16" s="6">
         <v>12</v>
       </c>
-      <c r="N16" t="s">
+      <c r="O16" t="s">
         <v>69</v>
       </c>
-      <c r="O16" s="4" t="s">
+      <c r="P16" s="4" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A17" s="6">
         <v>10</v>
       </c>
@@ -1231,17 +1258,17 @@
       <c r="C17" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="M17" s="6">
+      <c r="N17" s="6">
         <v>13</v>
       </c>
-      <c r="N17" t="s">
+      <c r="O17" t="s">
         <v>70</v>
       </c>
-      <c r="O17" s="4" t="s">
+      <c r="P17" s="4" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A18" s="6">
         <v>11</v>
       </c>
@@ -1251,17 +1278,17 @@
       <c r="C18" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="M18" s="6">
+      <c r="N18" s="6">
         <v>14</v>
       </c>
-      <c r="N18" t="s">
+      <c r="O18" t="s">
         <v>71</v>
       </c>
-      <c r="O18" s="4" t="s">
+      <c r="P18" s="4" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A19" s="6">
         <v>12</v>
       </c>
@@ -1271,17 +1298,17 @@
       <c r="C19" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="M19" s="6">
+      <c r="N19" s="6">
         <v>15</v>
       </c>
-      <c r="N19" t="s">
+      <c r="O19" t="s">
         <v>72</v>
       </c>
-      <c r="O19" s="4" t="s">
+      <c r="P19" s="4" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A20" s="6">
         <v>13</v>
       </c>
@@ -1291,17 +1318,17 @@
       <c r="C20" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="M20" s="6">
+      <c r="N20" s="6">
         <v>16</v>
       </c>
-      <c r="N20" t="s">
+      <c r="O20" t="s">
         <v>73</v>
       </c>
-      <c r="O20" s="4" t="s">
+      <c r="P20" s="4" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A21" s="6">
         <v>14</v>
       </c>
@@ -1311,17 +1338,17 @@
       <c r="C21" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="M21" s="6">
+      <c r="N21" s="6">
         <v>17</v>
       </c>
-      <c r="N21" t="s">
+      <c r="O21" t="s">
         <v>74</v>
       </c>
-      <c r="O21" s="4" t="s">
+      <c r="P21" s="4" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A22" s="6">
         <v>15</v>
       </c>
@@ -1331,31 +1358,31 @@
       <c r="C22" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="M22" s="6">
+      <c r="N22" s="6">
         <v>18</v>
       </c>
-      <c r="N22" t="s">
+      <c r="O22" t="s">
         <v>75</v>
       </c>
-      <c r="O22" s="3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P22" s="3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="23" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A23" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="M23" s="6">
+      <c r="N23" s="6">
         <v>19</v>
       </c>
-      <c r="N23" t="s">
+      <c r="O23" t="s">
         <v>76</v>
       </c>
-      <c r="O23" s="3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P23" s="3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="24" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A24" s="6">
         <v>16</v>
       </c>
@@ -1366,7 +1393,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A25" s="6">
         <v>17</v>
       </c>
@@ -1377,7 +1404,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A26" s="6">
         <v>18</v>
       </c>
@@ -1388,7 +1415,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A27" s="6">
         <v>19</v>
       </c>
@@ -1399,7 +1426,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A28" s="6">
         <v>20</v>
       </c>
@@ -1410,12 +1437,12 @@
         <v>89</v>
       </c>
     </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A29" s="6" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A30" s="7" t="s">
         <v>50</v>
       </c>
@@ -1426,7 +1453,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A31" s="7" t="s">
         <v>51</v>
       </c>
@@ -1437,7 +1464,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A32" s="9" t="s">
         <v>52</v>
       </c>
@@ -1504,8 +1531,9 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
     <mergeCell ref="A3:C3"/>
+    <mergeCell ref="I2:J2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Updated booklet week 8
Mostly updated week 8 and cleaned up some tables.
</commit_message>
<xml_diff>
--- a/course_revision_progress.xlsx
+++ b/course_revision_progress.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dhasterok/Documents/GitHub/EART_3017/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD7539E8-8B0F-BA47-AB87-A8405C5D74BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17435ABD-260C-4A4C-AE20-65F3E212077A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3100" yWindow="3400" windowWidth="26040" windowHeight="14680" xr2:uid="{4DB3ECE9-6214-0C48-84B8-5529643C9A33}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029" concurrentCalc="0"/>
+  <calcPr calcId="191029" concurrentCalc="0"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -871,8 +871,8 @@
       <c r="H6" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="I6" s="2" t="s">
-        <v>7</v>
+      <c r="I6" s="1" t="s">
+        <v>5</v>
       </c>
       <c r="J6" s="2"/>
       <c r="K6" s="2" t="s">
@@ -910,8 +910,8 @@
       <c r="H7" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="I7" s="2" t="s">
-        <v>7</v>
+      <c r="I7" s="1" t="s">
+        <v>5</v>
       </c>
       <c r="J7" s="2"/>
       <c r="K7" s="2" t="s">
@@ -976,8 +976,8 @@
       <c r="H9" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="I9" s="2" t="s">
-        <v>7</v>
+      <c r="I9" s="1" t="s">
+        <v>5</v>
       </c>
       <c r="J9" s="2"/>
       <c r="K9" s="2" t="s">
@@ -1015,8 +1015,8 @@
       <c r="H10" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="I10" s="2" t="s">
-        <v>7</v>
+      <c r="I10" s="1" t="s">
+        <v>5</v>
       </c>
       <c r="J10" s="2"/>
       <c r="K10" s="2" t="s">
@@ -1054,8 +1054,8 @@
       <c r="H11" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="I11" s="2" t="s">
-        <v>7</v>
+      <c r="I11" s="1" t="s">
+        <v>5</v>
       </c>
       <c r="J11" s="2"/>
       <c r="K11" s="2" t="s">
@@ -1087,8 +1087,8 @@
       <c r="H12" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="I12" s="2" t="s">
-        <v>7</v>
+      <c r="I12" s="1" t="s">
+        <v>5</v>
       </c>
       <c r="J12" s="2"/>
       <c r="K12" s="2" t="s">

</xml_diff>